<commit_message>
Update SGRE numbers to Q3 FY26 and add intelligence layer
- Siemens Energy segment results for Siemens Gamesa (FY24 - Q3 FY26): orders, revenue,
  profit before special items, service revenue, backlog, FY26 guidance
- Workbook with the 2026 order sheet; steel and copper series refreshed to October 2026
- New intel package: Executive Briefing and Intelligence Lab tabs, fiscal-year scenarios,
  announced-vs-reported comparison, data-quality checks, findings generator
- Tools for market refresh and cache rebuild; pytest suite; README
</commit_message>
<xml_diff>
--- a/SG_data_new.xlsx
+++ b/SG_data_new.xlsx
@@ -1,33 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr checkCompatibility="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\forsk\Documents\python\SGRE_sales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19737FA9-D022-4023-971D-ED222E9B71DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80CC344-5016-4E83-9394-997FD5EC3D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27300" yWindow="1380" windowWidth="20835" windowHeight="19410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3765" yWindow="1005" windowWidth="22575" windowHeight="18660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="economy" sheetId="2" r:id="rId1"/>
-    <sheet name="2025" sheetId="16" r:id="rId2"/>
-    <sheet name="2024" sheetId="15" r:id="rId3"/>
-    <sheet name="2023" sheetId="11" r:id="rId4"/>
-    <sheet name="2022" sheetId="3" r:id="rId5"/>
-    <sheet name="2021" sheetId="4" r:id="rId6"/>
-    <sheet name="2020" sheetId="5" r:id="rId7"/>
-    <sheet name="2019" sheetId="12" r:id="rId8"/>
-    <sheet name="2018" sheetId="13" r:id="rId9"/>
-    <sheet name="2017" sheetId="14" r:id="rId10"/>
-    <sheet name="projections" sheetId="10" r:id="rId11"/>
-    <sheet name="plots" sheetId="6" r:id="rId12"/>
-    <sheet name="delivery 2023" sheetId="7" r:id="rId13"/>
-    <sheet name="delivery 2024" sheetId="8" r:id="rId14"/>
-    <sheet name="delivery 2025" sheetId="9" r:id="rId15"/>
+    <sheet name="2026" sheetId="17" r:id="rId2"/>
+    <sheet name="2025" sheetId="16" r:id="rId3"/>
+    <sheet name="2024" sheetId="15" r:id="rId4"/>
+    <sheet name="2023" sheetId="11" r:id="rId5"/>
+    <sheet name="2022" sheetId="3" r:id="rId6"/>
+    <sheet name="2021" sheetId="4" r:id="rId7"/>
+    <sheet name="2020" sheetId="5" r:id="rId8"/>
+    <sheet name="2019" sheetId="12" r:id="rId9"/>
+    <sheet name="2018" sheetId="13" r:id="rId10"/>
+    <sheet name="2017" sheetId="14" r:id="rId11"/>
+    <sheet name="projections" sheetId="10" r:id="rId12"/>
+    <sheet name="plots" sheetId="6" r:id="rId13"/>
+    <sheet name="delivery 2023" sheetId="7" r:id="rId14"/>
+    <sheet name="delivery 2024" sheetId="8" r:id="rId15"/>
+    <sheet name="delivery 2025" sheetId="9" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1278" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="626">
   <si>
     <t>date</t>
   </si>
@@ -1904,6 +1905,30 @@
   </si>
   <si>
     <t>Total order offshore(€m)</t>
+  </si>
+  <si>
+    <t>SG 4.3-130</t>
+  </si>
+  <si>
+    <t>SG 7.0-170</t>
+  </si>
+  <si>
+    <t>Yinson Renewables</t>
+  </si>
+  <si>
+    <t>GETEC green energy</t>
+  </si>
+  <si>
+    <t>Stadtwerke Münster</t>
+  </si>
+  <si>
+    <t>Wind farm expected to generate over 300 GWh annually once operational</t>
+  </si>
+  <si>
+    <t>First SG 7.0-170 orders in Germany; article notes combined installation and maintenance</t>
+  </si>
+  <si>
+    <t>Expected annual production of 130 GWh; 6 turbines 250 m tall; will power ~42,000 households</t>
   </si>
 </sst>
 </file>
@@ -2080,7 +2105,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2118,6 +2143,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -6263,6 +6293,1175 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D487CCE4-9D3F-43CC-9D75-D425FB7A8A87}">
+  <dimension ref="B1:U35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="L1" s="23" t="s">
+        <v>290</v>
+      </c>
+      <c r="M1" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="N1" s="23" t="s">
+        <v>292</v>
+      </c>
+      <c r="O1" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="R1" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="S1" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="T1" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>530</v>
+      </c>
+      <c r="C2" t="s">
+        <v>329</v>
+      </c>
+      <c r="D2">
+        <v>200</v>
+      </c>
+      <c r="P2" t="s">
+        <v>330</v>
+      </c>
+      <c r="R2">
+        <v>2021</v>
+      </c>
+      <c r="S2" t="s">
+        <v>331</v>
+      </c>
+      <c r="U2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>531</v>
+      </c>
+      <c r="C3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D3">
+        <v>249</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>333</v>
+      </c>
+      <c r="I3">
+        <v>145</v>
+      </c>
+      <c r="J3">
+        <v>4.5</v>
+      </c>
+      <c r="S3" t="s">
+        <v>334</v>
+      </c>
+      <c r="U3" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>532</v>
+      </c>
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4">
+        <v>34.6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I4">
+        <v>132</v>
+      </c>
+      <c r="J4">
+        <v>3.4</v>
+      </c>
+      <c r="P4" t="s">
+        <v>336</v>
+      </c>
+      <c r="R4">
+        <v>2019</v>
+      </c>
+      <c r="S4" t="s">
+        <v>337</v>
+      </c>
+      <c r="U4" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>533</v>
+      </c>
+      <c r="C5" t="s">
+        <v>339</v>
+      </c>
+      <c r="D5">
+        <v>487</v>
+      </c>
+      <c r="E5">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5">
+        <v>167</v>
+      </c>
+      <c r="J5">
+        <v>8</v>
+      </c>
+      <c r="L5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M5">
+        <v>167</v>
+      </c>
+      <c r="N5">
+        <v>8</v>
+      </c>
+      <c r="P5" t="s">
+        <v>340</v>
+      </c>
+      <c r="R5">
+        <v>2020</v>
+      </c>
+      <c r="S5" t="s">
+        <v>341</v>
+      </c>
+      <c r="U5" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6">
+        <v>263</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="G6">
+        <v>34</v>
+      </c>
+      <c r="P6" t="s">
+        <v>343</v>
+      </c>
+      <c r="R6">
+        <v>2019</v>
+      </c>
+      <c r="S6" t="s">
+        <v>344</v>
+      </c>
+      <c r="U6" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>535</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7">
+        <v>176.8</v>
+      </c>
+      <c r="H7" t="s">
+        <v>346</v>
+      </c>
+      <c r="I7">
+        <v>122</v>
+      </c>
+      <c r="J7">
+        <v>2.1</v>
+      </c>
+      <c r="L7" t="s">
+        <v>347</v>
+      </c>
+      <c r="M7">
+        <v>114</v>
+      </c>
+      <c r="N7">
+        <v>2</v>
+      </c>
+      <c r="P7" t="s">
+        <v>348</v>
+      </c>
+      <c r="S7" t="s">
+        <v>349</v>
+      </c>
+      <c r="U7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>536</v>
+      </c>
+      <c r="C8" t="s">
+        <v>351</v>
+      </c>
+      <c r="D8">
+        <v>198.5</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+      <c r="G8">
+        <v>484</v>
+      </c>
+      <c r="H8" t="s">
+        <v>169</v>
+      </c>
+      <c r="I8">
+        <v>132</v>
+      </c>
+      <c r="J8">
+        <v>3.4</v>
+      </c>
+      <c r="L8" t="s">
+        <v>352</v>
+      </c>
+      <c r="M8">
+        <v>108</v>
+      </c>
+      <c r="N8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="P8" t="s">
+        <v>353</v>
+      </c>
+      <c r="S8" t="s">
+        <v>354</v>
+      </c>
+      <c r="U8" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>537</v>
+      </c>
+      <c r="C9" t="s">
+        <v>329</v>
+      </c>
+      <c r="D9">
+        <v>90</v>
+      </c>
+      <c r="G9">
+        <v>26</v>
+      </c>
+      <c r="H9" t="s">
+        <v>169</v>
+      </c>
+      <c r="I9">
+        <v>132</v>
+      </c>
+      <c r="J9">
+        <v>3.4</v>
+      </c>
+      <c r="P9" t="s">
+        <v>356</v>
+      </c>
+      <c r="R9">
+        <v>2020</v>
+      </c>
+      <c r="S9" t="s">
+        <v>357</v>
+      </c>
+      <c r="U9" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>538</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <v>120</v>
+      </c>
+      <c r="H10" t="s">
+        <v>359</v>
+      </c>
+      <c r="I10">
+        <v>154</v>
+      </c>
+      <c r="J10">
+        <v>6</v>
+      </c>
+      <c r="L10" t="s">
+        <v>28</v>
+      </c>
+      <c r="M10">
+        <v>167</v>
+      </c>
+      <c r="N10">
+        <v>8</v>
+      </c>
+      <c r="P10" t="s">
+        <v>360</v>
+      </c>
+      <c r="R10">
+        <v>2019</v>
+      </c>
+      <c r="S10" t="s">
+        <v>361</v>
+      </c>
+      <c r="U10" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>539</v>
+      </c>
+      <c r="C11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11">
+        <v>233</v>
+      </c>
+      <c r="G11">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>169</v>
+      </c>
+      <c r="I11">
+        <v>132</v>
+      </c>
+      <c r="J11">
+        <v>3.4</v>
+      </c>
+      <c r="L11" t="s">
+        <v>363</v>
+      </c>
+      <c r="M11">
+        <v>114</v>
+      </c>
+      <c r="N11">
+        <v>2.1</v>
+      </c>
+      <c r="P11" t="s">
+        <v>364</v>
+      </c>
+      <c r="S11" t="s">
+        <v>365</v>
+      </c>
+      <c r="U11" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>540</v>
+      </c>
+      <c r="C12" t="s">
+        <v>367</v>
+      </c>
+      <c r="D12">
+        <v>208</v>
+      </c>
+      <c r="G12">
+        <v>70</v>
+      </c>
+      <c r="P12" t="s">
+        <v>368</v>
+      </c>
+      <c r="R12">
+        <v>2019</v>
+      </c>
+      <c r="S12" t="s">
+        <v>369</v>
+      </c>
+      <c r="U12" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>541</v>
+      </c>
+      <c r="C13" t="s">
+        <v>351</v>
+      </c>
+      <c r="D13">
+        <v>4712</v>
+      </c>
+      <c r="H13" t="s">
+        <v>359</v>
+      </c>
+      <c r="I13">
+        <v>154</v>
+      </c>
+      <c r="J13">
+        <v>6</v>
+      </c>
+      <c r="P13" t="s">
+        <v>371</v>
+      </c>
+      <c r="R13">
+        <v>2020</v>
+      </c>
+      <c r="S13" t="s">
+        <v>372</v>
+      </c>
+      <c r="U13" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>542</v>
+      </c>
+      <c r="C14" t="s">
+        <v>374</v>
+      </c>
+      <c r="D14">
+        <v>380</v>
+      </c>
+      <c r="G14">
+        <v>89</v>
+      </c>
+      <c r="P14" t="s">
+        <v>375</v>
+      </c>
+      <c r="R14">
+        <v>2021</v>
+      </c>
+      <c r="S14" t="s">
+        <v>376</v>
+      </c>
+      <c r="U14" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>543</v>
+      </c>
+      <c r="C15" t="s">
+        <v>378</v>
+      </c>
+      <c r="D15">
+        <v>250</v>
+      </c>
+      <c r="H15" t="s">
+        <v>352</v>
+      </c>
+      <c r="I15">
+        <v>108</v>
+      </c>
+      <c r="J15">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="P15" t="s">
+        <v>379</v>
+      </c>
+      <c r="R15">
+        <v>2018</v>
+      </c>
+      <c r="S15" t="s">
+        <v>380</v>
+      </c>
+      <c r="U15" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>544</v>
+      </c>
+      <c r="C16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16">
+        <v>289</v>
+      </c>
+      <c r="E16">
+        <v>10</v>
+      </c>
+      <c r="G16">
+        <v>92</v>
+      </c>
+      <c r="H16" t="s">
+        <v>382</v>
+      </c>
+      <c r="I16">
+        <v>114</v>
+      </c>
+      <c r="J16">
+        <v>2.6</v>
+      </c>
+      <c r="L16" t="s">
+        <v>169</v>
+      </c>
+      <c r="M16">
+        <v>132</v>
+      </c>
+      <c r="N16">
+        <v>3.4</v>
+      </c>
+      <c r="P16" t="s">
+        <v>383</v>
+      </c>
+      <c r="S16" t="s">
+        <v>384</v>
+      </c>
+      <c r="U16" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>545</v>
+      </c>
+      <c r="C17" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17">
+        <v>1386</v>
+      </c>
+      <c r="G17">
+        <v>165</v>
+      </c>
+      <c r="H17" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17">
+        <v>167</v>
+      </c>
+      <c r="J17">
+        <v>8</v>
+      </c>
+      <c r="L17" t="s">
+        <v>16</v>
+      </c>
+      <c r="M17">
+        <v>154</v>
+      </c>
+      <c r="N17">
+        <v>7</v>
+      </c>
+      <c r="P17" t="s">
+        <v>386</v>
+      </c>
+      <c r="R17">
+        <v>2022</v>
+      </c>
+      <c r="S17" t="s">
+        <v>387</v>
+      </c>
+      <c r="U17" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>546</v>
+      </c>
+      <c r="C18" t="s">
+        <v>184</v>
+      </c>
+      <c r="D18">
+        <v>471</v>
+      </c>
+      <c r="G18">
+        <v>136</v>
+      </c>
+      <c r="H18" t="s">
+        <v>169</v>
+      </c>
+      <c r="I18">
+        <v>132</v>
+      </c>
+      <c r="J18">
+        <v>3.4</v>
+      </c>
+      <c r="S18" t="s">
+        <v>389</v>
+      </c>
+      <c r="U18" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>547</v>
+      </c>
+      <c r="C19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D19">
+        <v>300</v>
+      </c>
+      <c r="E19">
+        <v>10</v>
+      </c>
+      <c r="G19">
+        <v>143</v>
+      </c>
+      <c r="H19" t="s">
+        <v>346</v>
+      </c>
+      <c r="I19">
+        <v>122</v>
+      </c>
+      <c r="J19">
+        <v>2.1</v>
+      </c>
+      <c r="P19" t="s">
+        <v>391</v>
+      </c>
+      <c r="R19">
+        <v>2019</v>
+      </c>
+      <c r="S19" t="s">
+        <v>392</v>
+      </c>
+      <c r="U19" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="20" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>548</v>
+      </c>
+      <c r="C20" t="s">
+        <v>351</v>
+      </c>
+      <c r="D20">
+        <v>508</v>
+      </c>
+      <c r="P20" t="s">
+        <v>394</v>
+      </c>
+      <c r="S20" t="s">
+        <v>395</v>
+      </c>
+      <c r="U20" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="21" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>549</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21">
+        <v>140</v>
+      </c>
+      <c r="H21" t="s">
+        <v>347</v>
+      </c>
+      <c r="I21">
+        <v>114</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+      <c r="R21">
+        <v>2018</v>
+      </c>
+      <c r="S21" t="s">
+        <v>397</v>
+      </c>
+      <c r="U21" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>550</v>
+      </c>
+      <c r="C22" t="s">
+        <v>351</v>
+      </c>
+      <c r="D22">
+        <v>77</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="H22" t="s">
+        <v>399</v>
+      </c>
+      <c r="I22">
+        <v>120</v>
+      </c>
+      <c r="J22">
+        <v>2.625</v>
+      </c>
+      <c r="L22" t="s">
+        <v>352</v>
+      </c>
+      <c r="M22">
+        <v>108</v>
+      </c>
+      <c r="N22">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="P22" t="s">
+        <v>400</v>
+      </c>
+      <c r="R22">
+        <v>2018</v>
+      </c>
+      <c r="S22" t="s">
+        <v>401</v>
+      </c>
+      <c r="U22" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>551</v>
+      </c>
+      <c r="C23" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23">
+        <v>166</v>
+      </c>
+      <c r="H23" t="s">
+        <v>169</v>
+      </c>
+      <c r="I23">
+        <v>132</v>
+      </c>
+      <c r="J23">
+        <v>3.4</v>
+      </c>
+      <c r="R23">
+        <v>2019</v>
+      </c>
+      <c r="S23" t="s">
+        <v>403</v>
+      </c>
+      <c r="U23" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>552</v>
+      </c>
+      <c r="C24" t="s">
+        <v>405</v>
+      </c>
+      <c r="D24">
+        <v>194</v>
+      </c>
+      <c r="E24">
+        <v>25</v>
+      </c>
+      <c r="G24">
+        <v>56</v>
+      </c>
+      <c r="H24" t="s">
+        <v>169</v>
+      </c>
+      <c r="I24">
+        <v>132</v>
+      </c>
+      <c r="J24">
+        <v>3.4</v>
+      </c>
+      <c r="P24" t="s">
+        <v>406</v>
+      </c>
+      <c r="R24">
+        <v>2019</v>
+      </c>
+      <c r="S24" t="s">
+        <v>407</v>
+      </c>
+      <c r="U24" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>553</v>
+      </c>
+      <c r="C25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25">
+        <v>39</v>
+      </c>
+      <c r="G25">
+        <v>12</v>
+      </c>
+      <c r="H25" t="s">
+        <v>382</v>
+      </c>
+      <c r="I25">
+        <v>114</v>
+      </c>
+      <c r="J25">
+        <v>2.6</v>
+      </c>
+      <c r="P25" t="s">
+        <v>409</v>
+      </c>
+      <c r="R25">
+        <v>2020</v>
+      </c>
+      <c r="S25" t="s">
+        <v>410</v>
+      </c>
+      <c r="U25" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>554</v>
+      </c>
+      <c r="C26" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26">
+        <v>18</v>
+      </c>
+      <c r="H26" t="s">
+        <v>382</v>
+      </c>
+      <c r="I26">
+        <v>114</v>
+      </c>
+      <c r="J26">
+        <v>2.6</v>
+      </c>
+      <c r="P26" t="s">
+        <v>32</v>
+      </c>
+      <c r="S26" t="s">
+        <v>412</v>
+      </c>
+      <c r="U26" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>555</v>
+      </c>
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27">
+        <v>104</v>
+      </c>
+      <c r="E27">
+        <v>20</v>
+      </c>
+      <c r="F27" t="s">
+        <v>414</v>
+      </c>
+      <c r="G27">
+        <v>39</v>
+      </c>
+      <c r="H27" t="s">
+        <v>415</v>
+      </c>
+      <c r="I27">
+        <v>113</v>
+      </c>
+      <c r="J27">
+        <v>3.2</v>
+      </c>
+      <c r="L27" t="s">
+        <v>363</v>
+      </c>
+      <c r="M27">
+        <v>114</v>
+      </c>
+      <c r="N27">
+        <v>2.1</v>
+      </c>
+      <c r="P27" t="s">
+        <v>416</v>
+      </c>
+      <c r="Q27">
+        <v>3</v>
+      </c>
+      <c r="R27">
+        <v>2018</v>
+      </c>
+      <c r="S27" t="s">
+        <v>417</v>
+      </c>
+      <c r="U27" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>556</v>
+      </c>
+      <c r="C28" t="s">
+        <v>264</v>
+      </c>
+      <c r="G28">
+        <v>5</v>
+      </c>
+      <c r="S28" t="s">
+        <v>419</v>
+      </c>
+      <c r="U28" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>557</v>
+      </c>
+      <c r="C29" t="s">
+        <v>325</v>
+      </c>
+      <c r="D29">
+        <v>1000</v>
+      </c>
+      <c r="E29">
+        <v>15</v>
+      </c>
+      <c r="S29" t="s">
+        <v>421</v>
+      </c>
+      <c r="U29" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>558</v>
+      </c>
+      <c r="C30" t="s">
+        <v>423</v>
+      </c>
+      <c r="D30">
+        <v>36</v>
+      </c>
+      <c r="G30">
+        <v>18</v>
+      </c>
+      <c r="P30" t="s">
+        <v>424</v>
+      </c>
+      <c r="S30" t="s">
+        <v>425</v>
+      </c>
+      <c r="U30" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>559</v>
+      </c>
+      <c r="C31" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31">
+        <v>326</v>
+      </c>
+      <c r="R31">
+        <v>2018</v>
+      </c>
+      <c r="S31" t="s">
+        <v>427</v>
+      </c>
+      <c r="U31" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="32" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>560</v>
+      </c>
+      <c r="D32">
+        <v>330</v>
+      </c>
+      <c r="E32">
+        <v>10</v>
+      </c>
+      <c r="P32" t="s">
+        <v>429</v>
+      </c>
+      <c r="R32">
+        <v>2019</v>
+      </c>
+      <c r="S32" t="s">
+        <v>430</v>
+      </c>
+      <c r="U32" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="33" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>561</v>
+      </c>
+      <c r="C33" t="s">
+        <v>264</v>
+      </c>
+      <c r="D33">
+        <v>96</v>
+      </c>
+      <c r="P33" t="s">
+        <v>432</v>
+      </c>
+      <c r="R33">
+        <v>2018</v>
+      </c>
+      <c r="S33" t="s">
+        <v>433</v>
+      </c>
+      <c r="U33" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="34" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>562</v>
+      </c>
+      <c r="C34" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34">
+        <v>500</v>
+      </c>
+      <c r="H34" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34">
+        <v>167</v>
+      </c>
+      <c r="J34">
+        <v>8</v>
+      </c>
+      <c r="L34" t="s">
+        <v>16</v>
+      </c>
+      <c r="M34">
+        <v>154</v>
+      </c>
+      <c r="N34">
+        <v>7</v>
+      </c>
+      <c r="P34" t="s">
+        <v>435</v>
+      </c>
+      <c r="S34" t="s">
+        <v>436</v>
+      </c>
+      <c r="U34" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="35" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>563</v>
+      </c>
+      <c r="C35" t="s">
+        <v>438</v>
+      </c>
+      <c r="D35">
+        <v>262</v>
+      </c>
+      <c r="E35">
+        <v>15</v>
+      </c>
+      <c r="F35" t="s">
+        <v>414</v>
+      </c>
+      <c r="P35" t="s">
+        <v>439</v>
+      </c>
+      <c r="R35">
+        <v>2026</v>
+      </c>
+      <c r="S35" t="s">
+        <v>440</v>
+      </c>
+      <c r="U35" t="s">
+        <v>441</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F67B05D-93E5-4954-81A1-49B38898A4E2}">
   <dimension ref="B1:U12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6614,7 +7813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CB991BD-C5D4-41D1-B259-D107731B8821}">
   <dimension ref="C1:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6944,7 +8143,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="C4:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7056,7 +8255,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6FB178-5E3A-496C-B9B8-F416FBA0C05E}">
   <dimension ref="A1:X30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7767,7 +8966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8A15C2-697B-4293-A9F2-853903645001}">
   <dimension ref="A1:X30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8420,7 +9619,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3896A3-3E70-4E2B-93C7-367C467AFDE4}">
   <dimension ref="A1:X30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8697,6 +9896,629 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A587FAC5-E606-47BF-9D53-09E392A6A2D3}">
+  <dimension ref="A1:X44"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.85546875" customWidth="1"/>
+    <col min="10" max="11" width="4.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.85546875" customWidth="1"/>
+    <col min="19" max="19" width="37.5703125" customWidth="1"/>
+    <col min="21" max="21" width="9.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="L1" s="23" t="s">
+        <v>290</v>
+      </c>
+      <c r="M1" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="N1" s="23" t="s">
+        <v>292</v>
+      </c>
+      <c r="O1" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="R1" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="S1" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="T1" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="V1" s="1"/>
+      <c r="X1" s="1"/>
+    </row>
+    <row r="2" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B2" s="2">
+        <v>46059</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2" s="36">
+        <v>94.6</v>
+      </c>
+      <c r="F2" s="38" t="s">
+        <v>620</v>
+      </c>
+      <c r="G2" s="37">
+        <v>22</v>
+      </c>
+      <c r="H2" s="36" t="s">
+        <v>618</v>
+      </c>
+      <c r="P2" s="24"/>
+      <c r="S2" s="39" t="s">
+        <v>623</v>
+      </c>
+      <c r="U2" s="6"/>
+    </row>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B3" s="2">
+        <v>46059</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="36">
+        <v>21</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>621</v>
+      </c>
+      <c r="G3" s="37">
+        <v>3</v>
+      </c>
+      <c r="H3" s="36" t="s">
+        <v>619</v>
+      </c>
+      <c r="P3" s="24"/>
+      <c r="S3" s="39" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
+        <v>46062</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="36">
+        <v>42</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>622</v>
+      </c>
+      <c r="G4" s="37">
+        <v>6</v>
+      </c>
+      <c r="H4" s="36" t="s">
+        <v>619</v>
+      </c>
+      <c r="P4" s="24"/>
+      <c r="S4" s="39" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B5" s="2"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="X5" s="6"/>
+    </row>
+    <row r="6" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B6" s="2"/>
+      <c r="D6" s="5"/>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B7" s="2"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B8" s="2"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B9" s="2"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B10" s="2"/>
+      <c r="D10" s="4"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B14" s="2"/>
+      <c r="D14" s="4"/>
+      <c r="G14" s="3"/>
+    </row>
+    <row r="15" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B15" s="2"/>
+      <c r="D15" s="4"/>
+      <c r="G15" s="3"/>
+    </row>
+    <row r="16" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+      <c r="D16" s="4"/>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="D17" s="4"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="D18" s="5"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="D19" s="5"/>
+      <c r="G19" s="3"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B20" s="2"/>
+      <c r="D20" s="5"/>
+      <c r="G20" s="3"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A22" s="24"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+      <c r="O22" s="24"/>
+      <c r="X22" s="6"/>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24"/>
+      <c r="N23" s="24"/>
+      <c r="O23" s="24"/>
+    </row>
+    <row r="24" spans="1:24" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="24">
+        <f>SUM(D2:D22)</f>
+        <v>157.6</v>
+      </c>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24"/>
+      <c r="N24" s="24"/>
+      <c r="O24" s="24"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="24"/>
+      <c r="N25" s="24"/>
+      <c r="O25" s="24"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24"/>
+      <c r="N26" s="24"/>
+      <c r="O26" s="24"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="O27" s="24"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A28" s="24"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="O28" s="24"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A29" s="24"/>
+      <c r="B29" s="34"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="31"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="24"/>
+      <c r="O29" s="24"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A30" s="24"/>
+      <c r="B30" s="34"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+      <c r="L30" s="31"/>
+      <c r="M30" s="31"/>
+      <c r="N30" s="24"/>
+      <c r="O30" s="24"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A31" s="24"/>
+      <c r="B31" s="34"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="24"/>
+      <c r="L31" s="31"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="24"/>
+      <c r="O31" s="24"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A32" s="24"/>
+      <c r="B32" s="34"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
+      <c r="L32" s="31"/>
+      <c r="M32" s="31"/>
+      <c r="N32" s="24"/>
+      <c r="O32" s="24"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="24"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" s="24"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="31"/>
+      <c r="M34" s="31"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="24"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="24"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
+      <c r="J35" s="24"/>
+      <c r="K35" s="24"/>
+      <c r="L35" s="31"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="24"/>
+      <c r="O35" s="24"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" s="24"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="24"/>
+      <c r="J36" s="24"/>
+      <c r="K36" s="24"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="24"/>
+      <c r="O36" s="24"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="30"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="24"/>
+      <c r="J37" s="24"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="31"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="24"/>
+      <c r="O37" s="24"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" s="24"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="24"/>
+      <c r="J38" s="24"/>
+      <c r="K38" s="24"/>
+      <c r="L38" s="24"/>
+      <c r="M38" s="24"/>
+      <c r="N38" s="24"/>
+      <c r="O38" s="24"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="30"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="24"/>
+      <c r="J39" s="24"/>
+      <c r="K39" s="24"/>
+      <c r="L39" s="24"/>
+      <c r="M39" s="24"/>
+      <c r="N39" s="24"/>
+      <c r="O39" s="24"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="30"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="24"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="24"/>
+      <c r="N40" s="24"/>
+      <c r="O40" s="24"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="24"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="30"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="24"/>
+      <c r="I41" s="24"/>
+      <c r="J41" s="24"/>
+      <c r="K41" s="24"/>
+      <c r="L41" s="24"/>
+      <c r="M41" s="24"/>
+      <c r="N41" s="24"/>
+      <c r="O41" s="24"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="30"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="24"/>
+      <c r="I42" s="24"/>
+      <c r="J42" s="24"/>
+      <c r="K42" s="24"/>
+      <c r="L42" s="24"/>
+      <c r="M42" s="24"/>
+      <c r="N42" s="24"/>
+      <c r="O42" s="24"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="24"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="24"/>
+      <c r="H43" s="24"/>
+      <c r="I43" s="24"/>
+      <c r="J43" s="24"/>
+      <c r="K43" s="24"/>
+      <c r="L43" s="24"/>
+      <c r="M43" s="24"/>
+      <c r="N43" s="24"/>
+      <c r="O43" s="24"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="24"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="24"/>
+      <c r="H44" s="24"/>
+      <c r="I44" s="24"/>
+      <c r="J44" s="24"/>
+      <c r="K44" s="24"/>
+      <c r="L44" s="24"/>
+      <c r="M44" s="24"/>
+      <c r="N44" s="24"/>
+      <c r="O44" s="24"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF2D719-BE2C-415B-9CC9-F97ABA843ABD}">
   <dimension ref="A1:X44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9342,7 +11164,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80E0F23-F4EB-4E80-824F-FA2B0C619DCA}">
   <dimension ref="A1:X44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9991,7 +11813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B759D9-F4B2-4E58-83CB-17F61BB4E768}">
   <dimension ref="A1:X46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10710,7 +12532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11881,7 +13703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13272,7 +15094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14701,7 +16523,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B254786-E2CF-4F8F-BCF2-3E604847C519}">
   <dimension ref="B1:U21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -15435,1173 +17257,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D487CCE4-9D3F-43CC-9D75-D425FB7A8A87}">
-  <dimension ref="B1:U35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B1" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="23" t="s">
-        <v>289</v>
-      </c>
-      <c r="L1" s="23" t="s">
-        <v>290</v>
-      </c>
-      <c r="M1" s="23" t="s">
-        <v>291</v>
-      </c>
-      <c r="N1" s="23" t="s">
-        <v>292</v>
-      </c>
-      <c r="O1" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="R1" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="S1" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="T1" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" s="23" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>530</v>
-      </c>
-      <c r="C2" t="s">
-        <v>329</v>
-      </c>
-      <c r="D2">
-        <v>200</v>
-      </c>
-      <c r="P2" t="s">
-        <v>330</v>
-      </c>
-      <c r="R2">
-        <v>2021</v>
-      </c>
-      <c r="S2" t="s">
-        <v>331</v>
-      </c>
-      <c r="U2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>531</v>
-      </c>
-      <c r="C3" t="s">
-        <v>322</v>
-      </c>
-      <c r="D3">
-        <v>249</v>
-      </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="H3" t="s">
-        <v>333</v>
-      </c>
-      <c r="I3">
-        <v>145</v>
-      </c>
-      <c r="J3">
-        <v>4.5</v>
-      </c>
-      <c r="S3" t="s">
-        <v>334</v>
-      </c>
-      <c r="U3" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>532</v>
-      </c>
-      <c r="C4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D4">
-        <v>34.6</v>
-      </c>
-      <c r="H4" t="s">
-        <v>169</v>
-      </c>
-      <c r="I4">
-        <v>132</v>
-      </c>
-      <c r="J4">
-        <v>3.4</v>
-      </c>
-      <c r="P4" t="s">
-        <v>336</v>
-      </c>
-      <c r="R4">
-        <v>2019</v>
-      </c>
-      <c r="S4" t="s">
-        <v>337</v>
-      </c>
-      <c r="U4" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>533</v>
-      </c>
-      <c r="C5" t="s">
-        <v>339</v>
-      </c>
-      <c r="D5">
-        <v>487</v>
-      </c>
-      <c r="E5">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5">
-        <v>167</v>
-      </c>
-      <c r="J5">
-        <v>8</v>
-      </c>
-      <c r="L5" t="s">
-        <v>79</v>
-      </c>
-      <c r="M5">
-        <v>167</v>
-      </c>
-      <c r="N5">
-        <v>8</v>
-      </c>
-      <c r="P5" t="s">
-        <v>340</v>
-      </c>
-      <c r="R5">
-        <v>2020</v>
-      </c>
-      <c r="S5" t="s">
-        <v>341</v>
-      </c>
-      <c r="U5" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>534</v>
-      </c>
-      <c r="C6" t="s">
-        <v>86</v>
-      </c>
-      <c r="D6">
-        <v>263</v>
-      </c>
-      <c r="E6">
-        <v>20</v>
-      </c>
-      <c r="G6">
-        <v>34</v>
-      </c>
-      <c r="P6" t="s">
-        <v>343</v>
-      </c>
-      <c r="R6">
-        <v>2019</v>
-      </c>
-      <c r="S6" t="s">
-        <v>344</v>
-      </c>
-      <c r="U6" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>535</v>
-      </c>
-      <c r="C7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7">
-        <v>176.8</v>
-      </c>
-      <c r="H7" t="s">
-        <v>346</v>
-      </c>
-      <c r="I7">
-        <v>122</v>
-      </c>
-      <c r="J7">
-        <v>2.1</v>
-      </c>
-      <c r="L7" t="s">
-        <v>347</v>
-      </c>
-      <c r="M7">
-        <v>114</v>
-      </c>
-      <c r="N7">
-        <v>2</v>
-      </c>
-      <c r="P7" t="s">
-        <v>348</v>
-      </c>
-      <c r="S7" t="s">
-        <v>349</v>
-      </c>
-      <c r="U7" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>536</v>
-      </c>
-      <c r="C8" t="s">
-        <v>351</v>
-      </c>
-      <c r="D8">
-        <v>198.5</v>
-      </c>
-      <c r="E8">
-        <v>20</v>
-      </c>
-      <c r="G8">
-        <v>484</v>
-      </c>
-      <c r="H8" t="s">
-        <v>169</v>
-      </c>
-      <c r="I8">
-        <v>132</v>
-      </c>
-      <c r="J8">
-        <v>3.4</v>
-      </c>
-      <c r="L8" t="s">
-        <v>352</v>
-      </c>
-      <c r="M8">
-        <v>108</v>
-      </c>
-      <c r="N8">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="P8" t="s">
-        <v>353</v>
-      </c>
-      <c r="S8" t="s">
-        <v>354</v>
-      </c>
-      <c r="U8" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>537</v>
-      </c>
-      <c r="C9" t="s">
-        <v>329</v>
-      </c>
-      <c r="D9">
-        <v>90</v>
-      </c>
-      <c r="G9">
-        <v>26</v>
-      </c>
-      <c r="H9" t="s">
-        <v>169</v>
-      </c>
-      <c r="I9">
-        <v>132</v>
-      </c>
-      <c r="J9">
-        <v>3.4</v>
-      </c>
-      <c r="P9" t="s">
-        <v>356</v>
-      </c>
-      <c r="R9">
-        <v>2020</v>
-      </c>
-      <c r="S9" t="s">
-        <v>357</v>
-      </c>
-      <c r="U9" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>538</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10">
-        <v>120</v>
-      </c>
-      <c r="H10" t="s">
-        <v>359</v>
-      </c>
-      <c r="I10">
-        <v>154</v>
-      </c>
-      <c r="J10">
-        <v>6</v>
-      </c>
-      <c r="L10" t="s">
-        <v>28</v>
-      </c>
-      <c r="M10">
-        <v>167</v>
-      </c>
-      <c r="N10">
-        <v>8</v>
-      </c>
-      <c r="P10" t="s">
-        <v>360</v>
-      </c>
-      <c r="R10">
-        <v>2019</v>
-      </c>
-      <c r="S10" t="s">
-        <v>361</v>
-      </c>
-      <c r="U10" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>539</v>
-      </c>
-      <c r="C11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11">
-        <v>233</v>
-      </c>
-      <c r="G11">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>169</v>
-      </c>
-      <c r="I11">
-        <v>132</v>
-      </c>
-      <c r="J11">
-        <v>3.4</v>
-      </c>
-      <c r="L11" t="s">
-        <v>363</v>
-      </c>
-      <c r="M11">
-        <v>114</v>
-      </c>
-      <c r="N11">
-        <v>2.1</v>
-      </c>
-      <c r="P11" t="s">
-        <v>364</v>
-      </c>
-      <c r="S11" t="s">
-        <v>365</v>
-      </c>
-      <c r="U11" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>540</v>
-      </c>
-      <c r="C12" t="s">
-        <v>367</v>
-      </c>
-      <c r="D12">
-        <v>208</v>
-      </c>
-      <c r="G12">
-        <v>70</v>
-      </c>
-      <c r="P12" t="s">
-        <v>368</v>
-      </c>
-      <c r="R12">
-        <v>2019</v>
-      </c>
-      <c r="S12" t="s">
-        <v>369</v>
-      </c>
-      <c r="U12" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>541</v>
-      </c>
-      <c r="C13" t="s">
-        <v>351</v>
-      </c>
-      <c r="D13">
-        <v>4712</v>
-      </c>
-      <c r="H13" t="s">
-        <v>359</v>
-      </c>
-      <c r="I13">
-        <v>154</v>
-      </c>
-      <c r="J13">
-        <v>6</v>
-      </c>
-      <c r="P13" t="s">
-        <v>371</v>
-      </c>
-      <c r="R13">
-        <v>2020</v>
-      </c>
-      <c r="S13" t="s">
-        <v>372</v>
-      </c>
-      <c r="U13" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>542</v>
-      </c>
-      <c r="C14" t="s">
-        <v>374</v>
-      </c>
-      <c r="D14">
-        <v>380</v>
-      </c>
-      <c r="G14">
-        <v>89</v>
-      </c>
-      <c r="P14" t="s">
-        <v>375</v>
-      </c>
-      <c r="R14">
-        <v>2021</v>
-      </c>
-      <c r="S14" t="s">
-        <v>376</v>
-      </c>
-      <c r="U14" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>543</v>
-      </c>
-      <c r="C15" t="s">
-        <v>378</v>
-      </c>
-      <c r="D15">
-        <v>250</v>
-      </c>
-      <c r="H15" t="s">
-        <v>352</v>
-      </c>
-      <c r="I15">
-        <v>108</v>
-      </c>
-      <c r="J15">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="P15" t="s">
-        <v>379</v>
-      </c>
-      <c r="R15">
-        <v>2018</v>
-      </c>
-      <c r="S15" t="s">
-        <v>380</v>
-      </c>
-      <c r="U15" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>544</v>
-      </c>
-      <c r="C16" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16">
-        <v>289</v>
-      </c>
-      <c r="E16">
-        <v>10</v>
-      </c>
-      <c r="G16">
-        <v>92</v>
-      </c>
-      <c r="H16" t="s">
-        <v>382</v>
-      </c>
-      <c r="I16">
-        <v>114</v>
-      </c>
-      <c r="J16">
-        <v>2.6</v>
-      </c>
-      <c r="L16" t="s">
-        <v>169</v>
-      </c>
-      <c r="M16">
-        <v>132</v>
-      </c>
-      <c r="N16">
-        <v>3.4</v>
-      </c>
-      <c r="P16" t="s">
-        <v>383</v>
-      </c>
-      <c r="S16" t="s">
-        <v>384</v>
-      </c>
-      <c r="U16" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>545</v>
-      </c>
-      <c r="C17" t="s">
-        <v>104</v>
-      </c>
-      <c r="D17">
-        <v>1386</v>
-      </c>
-      <c r="G17">
-        <v>165</v>
-      </c>
-      <c r="H17" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17">
-        <v>167</v>
-      </c>
-      <c r="J17">
-        <v>8</v>
-      </c>
-      <c r="L17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M17">
-        <v>154</v>
-      </c>
-      <c r="N17">
-        <v>7</v>
-      </c>
-      <c r="P17" t="s">
-        <v>386</v>
-      </c>
-      <c r="R17">
-        <v>2022</v>
-      </c>
-      <c r="S17" t="s">
-        <v>387</v>
-      </c>
-      <c r="U17" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>546</v>
-      </c>
-      <c r="C18" t="s">
-        <v>184</v>
-      </c>
-      <c r="D18">
-        <v>471</v>
-      </c>
-      <c r="G18">
-        <v>136</v>
-      </c>
-      <c r="H18" t="s">
-        <v>169</v>
-      </c>
-      <c r="I18">
-        <v>132</v>
-      </c>
-      <c r="J18">
-        <v>3.4</v>
-      </c>
-      <c r="S18" t="s">
-        <v>389</v>
-      </c>
-      <c r="U18" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>547</v>
-      </c>
-      <c r="C19" t="s">
-        <v>75</v>
-      </c>
-      <c r="D19">
-        <v>300</v>
-      </c>
-      <c r="E19">
-        <v>10</v>
-      </c>
-      <c r="G19">
-        <v>143</v>
-      </c>
-      <c r="H19" t="s">
-        <v>346</v>
-      </c>
-      <c r="I19">
-        <v>122</v>
-      </c>
-      <c r="J19">
-        <v>2.1</v>
-      </c>
-      <c r="P19" t="s">
-        <v>391</v>
-      </c>
-      <c r="R19">
-        <v>2019</v>
-      </c>
-      <c r="S19" t="s">
-        <v>392</v>
-      </c>
-      <c r="U19" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="20" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
-        <v>548</v>
-      </c>
-      <c r="C20" t="s">
-        <v>351</v>
-      </c>
-      <c r="D20">
-        <v>508</v>
-      </c>
-      <c r="P20" t="s">
-        <v>394</v>
-      </c>
-      <c r="S20" t="s">
-        <v>395</v>
-      </c>
-      <c r="U20" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="21" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>549</v>
-      </c>
-      <c r="C21" t="s">
-        <v>75</v>
-      </c>
-      <c r="D21">
-        <v>140</v>
-      </c>
-      <c r="H21" t="s">
-        <v>347</v>
-      </c>
-      <c r="I21">
-        <v>114</v>
-      </c>
-      <c r="J21">
-        <v>2</v>
-      </c>
-      <c r="R21">
-        <v>2018</v>
-      </c>
-      <c r="S21" t="s">
-        <v>397</v>
-      </c>
-      <c r="U21" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>550</v>
-      </c>
-      <c r="C22" t="s">
-        <v>351</v>
-      </c>
-      <c r="D22">
-        <v>77</v>
-      </c>
-      <c r="E22">
-        <v>5</v>
-      </c>
-      <c r="H22" t="s">
-        <v>399</v>
-      </c>
-      <c r="I22">
-        <v>120</v>
-      </c>
-      <c r="J22">
-        <v>2.625</v>
-      </c>
-      <c r="L22" t="s">
-        <v>352</v>
-      </c>
-      <c r="M22">
-        <v>108</v>
-      </c>
-      <c r="N22">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="P22" t="s">
-        <v>400</v>
-      </c>
-      <c r="R22">
-        <v>2018</v>
-      </c>
-      <c r="S22" t="s">
-        <v>401</v>
-      </c>
-      <c r="U22" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>551</v>
-      </c>
-      <c r="C23" t="s">
-        <v>88</v>
-      </c>
-      <c r="D23">
-        <v>166</v>
-      </c>
-      <c r="H23" t="s">
-        <v>169</v>
-      </c>
-      <c r="I23">
-        <v>132</v>
-      </c>
-      <c r="J23">
-        <v>3.4</v>
-      </c>
-      <c r="R23">
-        <v>2019</v>
-      </c>
-      <c r="S23" t="s">
-        <v>403</v>
-      </c>
-      <c r="U23" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>552</v>
-      </c>
-      <c r="C24" t="s">
-        <v>405</v>
-      </c>
-      <c r="D24">
-        <v>194</v>
-      </c>
-      <c r="E24">
-        <v>25</v>
-      </c>
-      <c r="G24">
-        <v>56</v>
-      </c>
-      <c r="H24" t="s">
-        <v>169</v>
-      </c>
-      <c r="I24">
-        <v>132</v>
-      </c>
-      <c r="J24">
-        <v>3.4</v>
-      </c>
-      <c r="P24" t="s">
-        <v>406</v>
-      </c>
-      <c r="R24">
-        <v>2019</v>
-      </c>
-      <c r="S24" t="s">
-        <v>407</v>
-      </c>
-      <c r="U24" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>553</v>
-      </c>
-      <c r="C25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D25">
-        <v>39</v>
-      </c>
-      <c r="G25">
-        <v>12</v>
-      </c>
-      <c r="H25" t="s">
-        <v>382</v>
-      </c>
-      <c r="I25">
-        <v>114</v>
-      </c>
-      <c r="J25">
-        <v>2.6</v>
-      </c>
-      <c r="P25" t="s">
-        <v>409</v>
-      </c>
-      <c r="R25">
-        <v>2020</v>
-      </c>
-      <c r="S25" t="s">
-        <v>410</v>
-      </c>
-      <c r="U25" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>554</v>
-      </c>
-      <c r="C26" t="s">
-        <v>88</v>
-      </c>
-      <c r="D26">
-        <v>18</v>
-      </c>
-      <c r="H26" t="s">
-        <v>382</v>
-      </c>
-      <c r="I26">
-        <v>114</v>
-      </c>
-      <c r="J26">
-        <v>2.6</v>
-      </c>
-      <c r="P26" t="s">
-        <v>32</v>
-      </c>
-      <c r="S26" t="s">
-        <v>412</v>
-      </c>
-      <c r="U26" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>555</v>
-      </c>
-      <c r="C27" t="s">
-        <v>19</v>
-      </c>
-      <c r="D27">
-        <v>104</v>
-      </c>
-      <c r="E27">
-        <v>20</v>
-      </c>
-      <c r="F27" t="s">
-        <v>414</v>
-      </c>
-      <c r="G27">
-        <v>39</v>
-      </c>
-      <c r="H27" t="s">
-        <v>415</v>
-      </c>
-      <c r="I27">
-        <v>113</v>
-      </c>
-      <c r="J27">
-        <v>3.2</v>
-      </c>
-      <c r="L27" t="s">
-        <v>363</v>
-      </c>
-      <c r="M27">
-        <v>114</v>
-      </c>
-      <c r="N27">
-        <v>2.1</v>
-      </c>
-      <c r="P27" t="s">
-        <v>416</v>
-      </c>
-      <c r="Q27">
-        <v>3</v>
-      </c>
-      <c r="R27">
-        <v>2018</v>
-      </c>
-      <c r="S27" t="s">
-        <v>417</v>
-      </c>
-      <c r="U27" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>556</v>
-      </c>
-      <c r="C28" t="s">
-        <v>264</v>
-      </c>
-      <c r="G28">
-        <v>5</v>
-      </c>
-      <c r="S28" t="s">
-        <v>419</v>
-      </c>
-      <c r="U28" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>557</v>
-      </c>
-      <c r="C29" t="s">
-        <v>325</v>
-      </c>
-      <c r="D29">
-        <v>1000</v>
-      </c>
-      <c r="E29">
-        <v>15</v>
-      </c>
-      <c r="S29" t="s">
-        <v>421</v>
-      </c>
-      <c r="U29" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>558</v>
-      </c>
-      <c r="C30" t="s">
-        <v>423</v>
-      </c>
-      <c r="D30">
-        <v>36</v>
-      </c>
-      <c r="G30">
-        <v>18</v>
-      </c>
-      <c r="P30" t="s">
-        <v>424</v>
-      </c>
-      <c r="S30" t="s">
-        <v>425</v>
-      </c>
-      <c r="U30" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>559</v>
-      </c>
-      <c r="C31" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31">
-        <v>326</v>
-      </c>
-      <c r="R31">
-        <v>2018</v>
-      </c>
-      <c r="S31" t="s">
-        <v>427</v>
-      </c>
-      <c r="U31" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="32" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>560</v>
-      </c>
-      <c r="D32">
-        <v>330</v>
-      </c>
-      <c r="E32">
-        <v>10</v>
-      </c>
-      <c r="P32" t="s">
-        <v>429</v>
-      </c>
-      <c r="R32">
-        <v>2019</v>
-      </c>
-      <c r="S32" t="s">
-        <v>430</v>
-      </c>
-      <c r="U32" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="33" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>561</v>
-      </c>
-      <c r="C33" t="s">
-        <v>264</v>
-      </c>
-      <c r="D33">
-        <v>96</v>
-      </c>
-      <c r="P33" t="s">
-        <v>432</v>
-      </c>
-      <c r="R33">
-        <v>2018</v>
-      </c>
-      <c r="S33" t="s">
-        <v>433</v>
-      </c>
-      <c r="U33" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="34" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>562</v>
-      </c>
-      <c r="C34" t="s">
-        <v>19</v>
-      </c>
-      <c r="D34">
-        <v>500</v>
-      </c>
-      <c r="H34" t="s">
-        <v>28</v>
-      </c>
-      <c r="I34">
-        <v>167</v>
-      </c>
-      <c r="J34">
-        <v>8</v>
-      </c>
-      <c r="L34" t="s">
-        <v>16</v>
-      </c>
-      <c r="M34">
-        <v>154</v>
-      </c>
-      <c r="N34">
-        <v>7</v>
-      </c>
-      <c r="P34" t="s">
-        <v>435</v>
-      </c>
-      <c r="S34" t="s">
-        <v>436</v>
-      </c>
-      <c r="U34" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="35" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>563</v>
-      </c>
-      <c r="C35" t="s">
-        <v>438</v>
-      </c>
-      <c r="D35">
-        <v>262</v>
-      </c>
-      <c r="E35">
-        <v>15</v>
-      </c>
-      <c r="F35" t="s">
-        <v>414</v>
-      </c>
-      <c r="P35" t="s">
-        <v>439</v>
-      </c>
-      <c r="R35">
-        <v>2026</v>
-      </c>
-      <c r="S35" t="s">
-        <v>440</v>
-      </c>
-      <c r="U35" t="s">
-        <v>441</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>